<commit_message>
ops(vevor): generate shared full feed and worker assets
</commit_message>
<xml_diff>
--- a/operations/vendor-source/vevor/2026-09-10/04_Elevation_VEVOR_Curated_Catalog_Working_Set_2026-09-10_PUBLIC_SAFE.xlsx
+++ b/operations/vendor-source/vevor/2026-09-10/04_Elevation_VEVOR_Curated_Catalog_Working_Set_2026-09-10_PUBLIC_SAFE.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>395</t>
+          <t>381</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -546,11 +546,11 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>89.90000000000001</v>
+        <v>80.91</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>89.90000000000001</v>
+        <v>80.91</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>168</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>164</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -690,11 +690,11 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>252.71</v>
+        <v>319.9</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
-        <v>252.71</v>
+        <v>319.9</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>138</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -762,11 +762,11 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>184.94</v>
+        <v>166.45</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
-        <v>184.94</v>
+        <v>166.45</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>483</t>
+          <t>432</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -834,11 +834,11 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>195.21</v>
+        <v>216.9</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
-        <v>195.21</v>
+        <v>216.9</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>286</t>
+          <t>285</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -906,11 +906,11 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>159.95</v>
+        <v>143.96</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>159.95</v>
+        <v>143.96</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -969,7 +969,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>129</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>17514</t>
+          <t>21202</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1050,11 +1050,11 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>78.90000000000001</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>78.90000000000001</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>297</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automotive &gt; Battery Charging Systems &gt; Car Battery Chargers &gt; RV Charger </t>
+          <t xml:space="preserve">Automotive &gt; Battery Charging Systems &gt; Car Battery Chargers &gt; Forklift and Scissor Lift Charger </t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2895</t>
+          <t>2848</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1194,11 +1194,11 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>31.41</v>
+        <v>34.9</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>31.41</v>
+        <v>34.9</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2526</t>
+          <t>2576</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>57</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>100</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>180</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1482,11 +1482,11 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>473.9</v>
+        <v>426.51</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>473.9</v>
+        <v>426.51</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>133</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1554,11 +1554,11 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>785.9</v>
+        <v>707.3099999999999</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
-        <v>785.9</v>
+        <v>707.3099999999999</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>8570</t>
+          <t>8097</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1698,11 +1698,11 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>115.51</v>
+        <v>101.06</v>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="n">
-        <v>115.51</v>
+        <v>101.06</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10310</t>
+          <t>11658</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1770,11 +1770,11 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>143.56</v>
+        <v>121.41</v>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
-        <v>143.56</v>
+        <v>121.41</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2440</t>
+          <t>2502</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>483</t>
+          <t>446</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1914,11 +1914,11 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>49.41</v>
+        <v>44.47</v>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>49.41</v>
+        <v>44.47</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>587</t>
+          <t>520</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1986,11 +1986,11 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>152.9</v>
+        <v>129.9</v>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
-        <v>152.9</v>
+        <v>129.9</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>397</t>
+          <t>389</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>1532</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>13088</t>
+          <t>13525</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2202,11 +2202,11 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>47.9</v>
+        <v>43.11</v>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>47.9</v>
+        <v>43.11</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2387</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>149</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>1129</t>
+          <t>996</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2418,11 +2418,11 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>413.9</v>
+        <v>372.51</v>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="n">
-        <v>413.9</v>
+        <v>372.51</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>482</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>525</t>
+          <t>433</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>878</t>
+          <t>862</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2634,11 +2634,11 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>189.99</v>
+        <v>186.58</v>
       </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="n">
-        <v>189.99</v>
+        <v>186.58</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>1912</t>
+          <t>1882</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2706,11 +2706,11 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>66.90000000000001</v>
+        <v>60.21</v>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>66.90000000000001</v>
+        <v>60.21</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>1723</t>
+          <t>1473</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2778,11 +2778,11 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>59.9</v>
+        <v>53.91</v>
       </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>59.9</v>
+        <v>53.91</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2674</t>
+          <t>2462</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>3056</t>
+          <t>2860</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>1628</t>
+          <t>1607</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>882</t>
+          <t>773</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2073</t>
+          <t>1551</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3138,11 +3138,11 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>284.9</v>
+        <v>256.41</v>
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>284.9</v>
+        <v>256.41</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2854</t>
+          <t>2759</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3210,11 +3210,11 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>88.11</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>88.11</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>329</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3282,11 +3282,11 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>128.9</v>
+        <v>116.01</v>
       </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>128.9</v>
+        <v>116.01</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>45</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3354,11 +3354,11 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>239.9</v>
+        <v>227.91</v>
       </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>239.9</v>
+        <v>227.91</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>21005</v>
+        <v>21152</v>
       </c>
     </row>
     <row r="4">
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15982</v>
+        <v>16006</v>
       </c>
     </row>
     <row r="5">

</xml_diff>